<commit_message>
Add selection column functionality and manual input support in student card system
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1016,6 +1016,14 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>SG-EDU-2026-0147</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>